<commit_message>
Daily construction lead update
</commit_message>
<xml_diff>
--- a/data/nyc_construction_leads.xlsx
+++ b/data/nyc_construction_leads.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,12 +488,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>225 BROADWAY, Manhattan</t>
+          <t>110 WEST   88 STREET, Manhattan</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -503,221 +503,229 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>225 BROADWAY COMPANY LP</t>
+          <t>110 WEST 88 ST LLC</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1835600</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M01159723-P1</t>
+          <t>M01444600-I1</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Installation of new sprinkler heads on Basement, Ground fl, Mezzanine, 005, 007, 009, 010, 012, 014, 015, 017, 034 floors. No change in use, egress or occupancy.</t>
+          <t>CONSTRUCT NEW FIVE-STORY, ONE-FAMILY DWELLING (R-3) WITH CELLAR AND ROOF BULKHEAD, AS SHOWN ON PLANS. LPC COFA-21-06277</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Alexander</t>
+          <t>JASON S.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Bomstein</t>
+          <t>HERTZ</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>343 EAST   28 STREET, Brooklyn</t>
+          <t>2441 MORRIS AVENUE, Bronx</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TUR CONTRACTING INC</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Plan Examiner Assignment</t>
         </is>
       </c>
       <c r="G3" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>171630</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>B01445755-I1</t>
+          <t>X01342047-S7</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>DUE TO FIRE INCIDENT INTERIOR RENOVATION WORK ACCORDING TO PLAN. NO CHANGE IN USE, Egress or Occupancy. SUBSEQUENT FILE FOR PLUMBING FILLED SEPARATELY.</t>
+          <t>FOUNDATION APPLICATION BEING FILED FOR NEW BUILDING.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>MANSUR</t>
+          <t>Hasees</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>AHMED</t>
+          <t>Qazi</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>320 WEST   87 STREET, Manhattan</t>
+          <t>33-15 BELL BOULEVARD, Queens</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Manhattan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3315 BELL LLC</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G4" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>78000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>M01432455-I1</t>
+          <t>Q01353566-S1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Renovation of Apt. 1CE on first floor.  Partition work per plans.  No change in use, egress or occupancy.  PL work will be filed subsequently.</t>
+          <t>INSTALLATION OF SOE AND FOUNDATION AS PER THE PLANS FILED HEREWITH. NO CHANGE IN USE, OCCUPANCY OR EGRESS.</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Vladimir</t>
+          <t>MEHDI</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Lukyanov-Cherny</t>
+          <t>GHAZI</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>360 CENTRAL PARK WEST, Manhattan</t>
+          <t>2616 HARWAY AVENUE, Brooklyn</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Manhattan</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G5" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>122750</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>M01343461-P1</t>
+          <t>B01207648-S9</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Interior renovation of existing apartment. No change in use, egress or occupancy.</t>
+          <t>INSTALLATION OF HEAVY-DUTY SIDEWALK SHED FOR NEW BUILDING CONSTRUCTION AS PER PLANS.  NO CHANGE IN USE OCCUPANCY OR EGRESS UNDER THIS APPLICATION.  SIDEWALK SHED SHALL COMPLY WITH CHAPTER 33 OF THE 2022 NYC BUILDING CODE.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>KAMRUL</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Gregory</t>
+          <t>AHSAN</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>87-41 PARSONS BOULEVARD, Queens</t>
+          <t>33-11 BELL BOULEVARD, Queens</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -727,113 +735,113 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>NYC SCHOOL CONSTRUCTION</t>
+          <t>3315 BELL LLC</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G6" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Q01422166-I1</t>
+          <t>Q01391484-S1</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>INSTALLATION OF NEW SIDEWALK SHED FOR PS 86Q AT 87-41 PARSONS BOULEVARD, QUEENS IN CONJUNCTION WITH ALT# Q01263129, Q01422165, Q01422170 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+          <t>INSTALLATION OF SOE AND FOUNDATION AS PER THE PLANS FILED HEREWITH. NO CHANGE IN USE, OCCUPANCY OR EGRESS.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>MEHDI</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>HASAN</t>
+          <t>GHAZI</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>New Building</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>27-12 2 STREET, Queens</t>
+          <t>1232A EAST  224 STREET, Bronx</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>star dust</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Permit Issued</t>
+          <t>Pending CPE/ACPE Assignment</t>
         </is>
       </c>
       <c r="G7" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Q01446421-I1</t>
+          <t>X01433548-I1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>dd</t>
+          <t>ERECT 3 STORY WITH CELLAR, 4 FAMILY BUILDING AS PER PLANS SUBMITTED. NEW CO TO BE OBTAINED.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Aimarana</t>
+          <t>SERDAR</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>CEYLAN</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>ALT-CO - New Building with Existing Elements to Remain</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>139-32 249 STREET, Queens</t>
+          <t>67-45 169 STREET, Queens</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -843,98 +851,98 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ewanchin International Inc.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending CPE/ACPE Assignment</t>
         </is>
       </c>
       <c r="G8" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>8000</t>
+          <t>1167332</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Q01445813-I1</t>
+          <t>Q01446486-I1</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Construct a temporary fence along the property line</t>
+          <t>VERTICAL AND HORIZONTAL EXTENSION OF EXISTING ONE FAMILY + ADU. OBTAIN NEW C OF O.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>KOJO</t>
+          <t>KAI</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>SIMPSON</t>
+          <t>HUANG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alteration</t>
+          <t>Full Demolition</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>27-12 2 STREET, Queens</t>
+          <t>485 FULTON STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>star dust</t>
+          <t>OWNERS REP</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Pending Plan Examiner Assignment</t>
         </is>
       </c>
       <c r="G9" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1000000</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Q01446389-I1</t>
+          <t>B01426676-I1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>dd</t>
+          <t>Full demolition to a four story building</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Aimarana</t>
+          <t>DUY</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>HOANG</t>
         </is>
       </c>
     </row>
@@ -949,50 +957,50 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>310 EAST    2 STREET, Manhattan</t>
+          <t>1430 SHORE DRIVE, Bronx</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Manhattan</t>
+          <t>Bronx</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KAHEN PROPERTIES</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G10" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>20000</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>M01441809-I1</t>
+          <t>X01372332-S2</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Minor repairs in parking space at cellar level. Floor crack repairs, spall repairs, installing vehicle barrier, ceiling holes repair, pipe penetration fire stopping. Repairs as per plans filed.</t>
+          <t>Erect temproary construction fence</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>FNU</t>
+          <t>Kenneth</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>LUQMAN</t>
+          <t>Koons</t>
         </is>
       </c>
     </row>
@@ -1007,50 +1015,50 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>27-12 2 STREET, Queens</t>
+          <t>166 WEST   18 STREET, Manhattan</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Manhattan</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>star dust</t>
+          <t>Douglas Elliman Property Management</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Plan Examiner Review</t>
+          <t>Pending CPE/ACPE Assignment</t>
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>162690</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Q01446389-P1</t>
+          <t>M01389555-S1</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>dd</t>
+          <t>PLUMBING WORK FOR PHB (PENTHOUSE APT), FILED IN CONJUNCTION WITH GENERAL CONSTRUCTION APPLICATION. ALL AS PER PLANS AND APPLICATIONS. NO CHANGE IN USE, EGRESS OR OCCUAPNCY.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Aimarana</t>
+          <t>Abdallah</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>Elcherbini</t>
         </is>
       </c>
     </row>
@@ -1065,50 +1073,50 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>27-12 2 STREET, Queens</t>
+          <t>400 WEST   63 STREET, Manhattan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Manhattan</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>star dust</t>
+          <t>WINDSOR COMMUNITIES</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending QA Assignment</t>
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Q01446399-I1</t>
+          <t>M01446526-I1</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Window Inspection</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Aimarana</t>
+          <t>GEORGE</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>COLE</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1131,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>87-41 PARSONS BOULEVARD, Queens</t>
+          <t>38-29 216 STREET, Queens</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1133,40 +1141,40 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>NYC SCHOOL CONSTRUCTION</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46249</v>
+        <v>46251</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>85500</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Q01422165-I1</t>
+          <t>Q01347227-P2</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>INSTALLATION OF TEMPORARY CONSTRUCTION FENCE FOR PS 86Q AT 87-41 PARSONS BOULEVARD, QUEENS IN CONJUNCTION WITH ALT# Q01263129, Q01422166, Q01422170  AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+          <t>File application in conjunction with GC application Q01347224.</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>ADEL</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>HASAN</t>
+          <t>SAGEER</t>
         </is>
       </c>
     </row>
@@ -1181,50 +1189,50 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>87-41 PARSONS BOULEVARD, Queens</t>
+          <t>256 EAST    9 STREET, Brooklyn</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>NYC SCHOOL CONSTRUCTION</t>
+          <t>SAS CONTRACTING CO, INC</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46249</v>
+        <v>46251</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Q01422170-I1</t>
+          <t>B01265664-P1</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>INSTALLATION OF PIPE SCAFFOLD FOR PS 86Q AT 87-41 PARSONS BOULEVARD, QUEENS IN CONJUNCTION WITH ALT# Q01263129, Q01422165, Q01422166 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+          <t>FILING FOR PLUMBING WORK TO RESOLVE VIOLATIONS 34747192K, 34900629M</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>HASAN</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
@@ -1239,50 +1247,50 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>193-41 MCLAUGHLIN AVENUE, Queens</t>
+          <t>119 WEST   71 STREET, Manhattan</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Manhattan</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CHOI</t>
+          <t>SEQUOIA PROPERTY MANAGEMENT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Pending Prof Cert QA Assignment</t>
+          <t>Plan Examiner Review</t>
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>73500</t>
+          <t>20000</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Q01217421-P2</t>
+          <t>M01440096-S2</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>INTERIOR RENOVATION OF EXISTING 2 STORY RESIDENTIAL BUILDING. NO CHANGE OF EGRESS, USE AND OCCUPANCY.</t>
+          <t>DEMOLITION AND REMOVALS OF PORTIONS OF EXISTING FINISHES AND NON-STRUCTURAL ELEMENTS. NO CHANGE IN OCCUPANY, USE OR EGRESS.</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Jonar</t>
+          <t>Anthony</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Madriaga</t>
+          <t>Farina</t>
         </is>
       </c>
     </row>
@@ -1297,173 +1305,177 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>27-12 2 STREET, Queens</t>
+          <t>188 EAST   70 STREET, Manhattan</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Queens</t>
+          <t>Manhattan</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>star dust</t>
+          <t>DOUGLAS ELLIMAN PROPERTY MANAGEMENT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Permit Issued</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Q01446424-I1</t>
+          <t>M01443002-I1</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>sdfgdfg</t>
+          <t>INSTALLATION OF TEMPORARY HEAVY DUTY SIDEWALK SHED AS PER PLANS. NO CHANGE IN USE, EGRESS OR OCCUPANCY. SIDEWALK SHED SHALL COMPLY WITH CHAPTER #33 OF 2022 THE NYC BUILDING CODE. LIVE LOAD 300PSF.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Aimarana</t>
+          <t>Charles</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>Davidson</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Full Demolition</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>27-12 2 STREET, Queens</t>
+          <t>60 RIVERSIDE DRIVE, Manhattan</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Queens</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>star dust</t>
-        </is>
-      </c>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Pending Plan Examiner Assignment</t>
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Q01446361-I1</t>
+          <t>M01406823-S1</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>asfsdg</t>
+          <t>PLUMBING WORK ASSOCIATED WITH THE APARTMENT COMBINATION AND INTERIOR ALTERATION OF THE EXISTING APARTMENT #8A WITH #8H ON THE 8TH FLOOR INCLUDING MODIFICATION OF FIXTURES, DRAIN, AND WATER/ SANITARY LINES. NO CHANGE TO THE USE, EGRESS, OR OCCUPANCY.</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Aimarana</t>
+          <t>ALEX</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>ALAIMO</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>No Work</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>32-21 PARSONS BOULEVARD, Queens</t>
+          <t>156 5 AVENUE, Brooklyn</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Queens</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>GREENBROOK PARTNERS</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Pending CPE/ACPE Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>25000</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Q01428655-I1</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
+          <t>B01432441-I1</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>The scope of work consists of interior renovation of a commercial space to build a Deli food service establishment, including a commercial kitchen. Replace the existing storefront.</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>SUNG HO</t>
+          <t>Mourad</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>SHIN</t>
+          <t>Kicha</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>No Work</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>47-46 11 STREET, Queens</t>
+          <t>54-15 BEACH CHANNEL DRIVE, Queens</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1471,150 +1483,3092 @@
           <t>Queens</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NYCHA</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Q01223538-P3</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
+          <t>Q01443654-I1</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 54-15 BEACH CHANNEL DRIVE,  QUEENS NY 11692 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Devang</t>
+          <t>WALIUR</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Shah</t>
+          <t>RAHMAN</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Full Demolition</t>
+          <t>Alteration</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23REAR HOWARD AVENUE, Staten Island</t>
+          <t>21 FLATBUSH AVENUE, Brooklyn</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Staten Island</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>SABOR FOOD MARKET</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Pending Plan Examiner Assignment</t>
+          <t>Pending Prof Cert QA Assignment</t>
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>12000</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>S01431713-I1</t>
+          <t>B01345373-I1</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Full demolition of rear building (detached garage) as per plan.</t>
+          <t>FILING TO INSTALL THE MARKET KITCHEN HOOD AND DUCTWORK AS PER PLANS.</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>RUSSELL</t>
+          <t>KAMRUL</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>DANCE III</t>
+          <t>AHSAN</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
+        <v>40</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>779 FRANKLIN AVENUE, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>24000</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>B01419457-S1</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>PLUMBING AND ASSOCIATE PIPE WORKS FOR THE SPA INTERIOR RENOVATION.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Ng</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>40</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>339 BEACH   54 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>NYCHA</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Q01443699-I1</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 339 BEACH 54 STREET, QUEENS NY 11692 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>WALIUR</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>40</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1020 WALTON AVENUE, Bronx</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Bronx</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MEDALLION REAL ESTATE</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>X01377741-I1</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>FACADE REPAIRS AND REPLACE DAMAGED LENTILS</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Baalbaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>40</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>240 EAST   38 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>NYU LANGONE HEALTH</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>30459.15</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>M01290343-P1</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>NYU LANGONE HEALTH - ACC 16 CARDIA REHAB RENO - MODIFICATIONS TO AN EXISTING SPRINKLER SYSTEM AS PER PLANS FILED HEREWITH. NO CHANGE IN USE, EGRESS, OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>RAHUL</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>TIKEKAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>40</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>492 HENRY STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>45000</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>B01200434-P1</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>INTERIOR RENOVATION OF OF APARTMENT 5J INCLUDING, REPLACEMENT OF WOOD STAIRS. NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Nicola</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Salerno</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>40</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>133 EAST   58 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>133 E. 58TH STREET, LLC</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>21060</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>M01429675-I1</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>SPRINKLER MODIFICATIONS FILED HEREWITH.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Tomas</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Bagdas</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>40</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>159-70 HARLEM RIVER DRIVE, Manhattan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>NEW YORK CITY HOUSING AUTHORITY</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Pending QA Assignment</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>M01436744-I1</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Suspended Scaffolding for Facade Restoration/Repair</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>SAEED</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>ANJUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>40</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>179 STANTON STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>9000</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>M01444695-I1</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF HEAVY-DUTY SIDEWALK SHED TO PAINT THE CORNICE AS PER PLANS.  NO CHANGE IN USE OCCUPANCY OR EGRESS UNDER THIS APPLICATION.  SIDEWALK SHED SHALL COMPLY WITH CHAPTER 33 OF THE 2022 NYC BUILDING CODE.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>KAMRUL</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>AHSAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>40</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>180 PARK ROW, Manhattan</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>90000</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>M01203462-P1</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Demolition of doors, fixtures and finishes. New partitions, fixtures, finishes, and doors.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Devin</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Mills</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>40</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>492 HENRY STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>B01200531-P1</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>MODIFICATION TO PLUMBING FIXTURES IN APT 5J FOR INTERIOR RENOVATION . NO CHANGE TO USE, EGRESS OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Nicola</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Salerno</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>40</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>21-11 BROADWAY, Queens</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MUSS DEVELOPMENT LLC</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Q01443086-I1</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF AN ILLUMINATED BUSINESS ACCESSORY SIGN . NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>JIN HWAN</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>CHO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>40</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8117 11 AVENUE, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>FEILE LLC</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>21000</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>B00656705-S1</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF TEM. PIPE SCAFFOLD FOR NEW BUILDING CONSTRUCTION AS PER PLANS. SCAFFOLD SHALL COMPLY WITH CH #33 OF THE 2022 NYC BUILDING CODE. NO CHANGE IN USE, OCCUPANCY OR EGRESS UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>KAMRUL</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AHSAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>40</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>52-37 39 AVENUE, Queens</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Q01443173-I1</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>APPLICATION FILED TO SOLELY SIGNOFF PRE BIS APPLICATION ALT 1061-80.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Dario</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Pasquariello</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>40</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>575 SIXTH AVENUE, Manhattan</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>13677</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>M01420738-I1</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Plumbing changes to retail space on part of the cellar as indicated on drawings.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ARSEN</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>ZAVLYANOV</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>40</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>133 EAST   58 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>133 E. 58TH STREET, LLC</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>87000</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>M01429674-I1</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Installation of new plumbing fixtures as shown on plans.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Tomas</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Bagdas</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>40</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>575 SIXTH AVENUE, Manhattan</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>42866.93</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>M01420736-I1</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Mechanical changes to retail space on part of the cellar as indicated on drawings.</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ARSEN</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>ZAVLYANOV</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>40</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1948 BRUCKNER BOULEVARD, Bronx</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Bronx</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>VOLK INDUSTRIAL SERVICES CORP</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>23000</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>X01355236-P3</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF TEMPORARY PLYWOOD FENCE AS PER PLANS DURING CONSTRUCTION. NO CHANGE IN USE, EGRESS OR OCCUPANCY. FENCE SHALL COMPLY WITH CHAPTER 33 OF NYC BUILDING CODE OF 2022.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>KAMRUL</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>AHSAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>40</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>334 BEACH   56 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>NYCHA</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Q01443601-I1</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 334 BEACH 56TH STREET, QUEENS, NY 11692 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>WALIUR</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>40</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>133 EAST   58 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>133 E. 58TH STREET, LLC</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>285000</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>M01425747-I1</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Insulation of AC units and ductwork as shown on plans.</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Tomas</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Bagdas</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>40</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>80-13 91 AVENUE, Queens</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Abo Habib, LLC</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>89700</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Q01443488-I1</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>INTERIOR RENOVATION INSIDE EXISTING (1) FAMILY RESIDENTIAL HOME. WORK WILL INCLUDE REMOVAL OF INTERIOR PARTITIONS, NEW PARTITIONS, REPLACE EXISTING FLOOR WITH NEW, AND INTERIOR FINISHES THROUGHOUT. WORK AS PER PLANS.</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Hardik</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Shah</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>159-30 HARLEM RIVER DRIVE, Manhattan</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>NEW YORK CITY HOUSING AUTHORITY</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Pending QA Assignment</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>M01436572-I1</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Suspended Scaffolding for Facade Restoration/Repair</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>SAEED</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>ANJUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1215 BEDFORD AVENUE, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MOKAFE TIMES SQUARE CORP</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>20000</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>B01427163-I1</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>FILING FOR MINOR EXTERIOR FACADE REPAIR TO ADDRESS ECB VIOLATION# 39186508M, REPAIR STUCCO CRACKS AT THE FRONT OF BUILDING, AROUND THE WINDOWS, ARCH, AND RIGHT-SIDE CORNERS. THIS FILING IN CONJUNCTION WITH SIDEWALK SHED DOB NOW APPLICATION# B01399402.</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Hardik</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Shah</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>637 PARK PLACE, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>B01413681-I1</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Hardik</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Shah</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>37-13 UNION STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2970</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Q01441077-I1</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF NEW BUSINESS ACCESSORY ILLUMINATED WALL SIGN. NO CHANGE IN USE, OCCUPANCY OR EGRESS.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>JIN HWAN</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>CHO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1552 BROADWAY, Manhattan</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>WHARTON PROPERTIES LLC</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2970</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>M01441483-I1</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF AN ILLUMINATED BUSINESS ACCESSORY SIGN . NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>JIN HWAN</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>CHO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>40</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>779 FRANKLIN AVENUE, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>60000</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>B01419457-I1</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>INSTALL INTERIOR NON-LOAD BEARING PARTITIONS FOR SPA ON THE GROUND FLOOR. NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Ng</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>40</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>560 WEST  235 STREET, Bronx</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Bronx</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>PARKOFF</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>X01426137-I1</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Hardik</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Shah</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>40</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>159-04 HARLEM RIVER DRIVE, Manhattan</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>NEW YORK CITY HOUSING AUTHORITY</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Pending QA Assignment</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>M01436761-I1</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Suspended Scaffolding for Facade Restoration/Repair</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>SAEED</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>ANJUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>40</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>156 5 AVENUE, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>GREENBROOK PARTNERS</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>B01432441-S1</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>The scope of work consists of installing a new ADA toilet, kitchen sinks, and floor drains. Make modifications to the existing gas lines to accommodate the new cooking equipment.</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Mourad</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Kicha</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>40</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>36 EAST   31 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>36 EAST 31 COMPANY</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>5400</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>M01419849-S3</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>APPLICATION FILED FOR SPRINKLER ADDITIONS/MODIFICATIONS ON THE 5TH FLOOR AS PER PLANS FILED HEREWITH. NO CHANGE IN USE, EGRESS, OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Robert</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>McGee</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>40</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2814 BROADWAY, Manhattan</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>M01438367-I1</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF AN ILLUMINATED BUSINESS ACCESSORY SIGN . NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>JIN HWAN</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>CHO</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>40</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>235 EAST   58 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>150700</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>M01376995-P2</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>RENO. OF EXISTING DUPLEX APARTMENT/ GROUND COMMERCIAL NEW PARITIONS-RECONSTRUCTION STAIRS IN EXISTING OPENING- FINISHES-FIXTURES-BATHROOMS- NEW KITCHEN LAYOUT/ APPLIANCES-WINDOWS-ACCESSORY ROOF TERR. -NEW LIGHTING-NO CHANGE TO EGRESS USE OR OCCUPANCY</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Alyssa</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Manfredonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>40</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>166 WEST   18 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Douglas Elliman Property Management</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>177480</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>M01389555-S2</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Mechanical work associated with renovation in penthouse apartment. No change in use, egress or occupancy. All as per plans and applications.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Abdallah</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Elcherbini</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>40</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>54-15 BEACH CHANNEL DRIVE, Queens</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>NYCHA</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Q01443645-I1</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF TEMPORARY CONSTRUCTION FENCE AT 54-15 BEACH CHANEL DRIVE, QUEENS NY 11692  AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>WALIUR</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>40</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>365 BEACH   54 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>NYCHA</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Q01443681-I1</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 365 BEACH 54 STREET,  QUEENS NY 11692 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>WALIUR</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>40</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>354 BEACH   56 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>NYCHA</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Q01443628-I1</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF NEW SIDEWALK SHED AT 354 BEACH 56 STREET, QUEENS NY 11692 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>WALIUR</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>40</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>339 BEACH   54 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>NYCHA</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Q01443690-I1</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF TEMPORARY CONSTRUCTION FENCE AT 339 BEACH 54TH STREET, QUEENS NY 11692 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>WALIUR</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>40</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>159-18 HARLEM RIVER DRIVE, Manhattan</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>NEW YORK CITY HOUSING AUTHORITY</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Pending QA Assignment</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>M01436746-I1</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Suspended Scaffolding for Facade Restoration/Repair</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>SAEED</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>ANJUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>40</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>36 EAST   31 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>36 EAST 31 COMPANY</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>17000</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>M01419849-S2</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>APPLICATION FILED FOR PLUMBING ADDITIONS/MODIFICATIONS ON THE 5TH FLOOR AS PER PLANS FILED HEREWITH. NO CHANGE IN USE, EGRESS, OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Robert</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>McGee</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>40</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>159 COLUMBUS AVENUE, Manhattan</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>THE BRODSKY ORGANIZATION</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G60" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>M01444236-I1</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>PROPOSED MULTI-FACED ILLUMINATED, NON FLASHING, ACCESSORY BUSINESS SIGN.  NO CHANGE IN USE EGRESS NOR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Nazzareno</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Callipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>40</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>3521 THIRD AVENUE, Bronx</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Bronx</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G61" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>18000</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>X01442449-I1</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>APPLICATION FOR PLUMBING WORK AT THE KITCHEN OF THIS DELI-GROCERY STORE USE GROUP 6 (U.G. 6), AS PER PLANS. NO CHANGE IN USE, EGRESS OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>VICTOR</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>MARTINEZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>40</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>365 BEACH   54 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>NYCHA</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Q01443669-I1</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF TEMPORARY CONSTRUCTION FENCE AT 365 BEACH 54 STREET, QUEENS NY 11692 AS INDICATED ON PLANS. THERE WILL BE NO CHANGE IN THE USE, EGRESS, OR OCCUPANCY UNDER THIS APPLICATION.</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>WALIUR</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>RAHMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>40</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1215 HERKIMER STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>31250</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>B01278137-S1</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>(1)- Remove and cap gas line; gas risers gas meters gas boiler and cooking range; (2)- Remove existing plumbing fixtures and replace with new plumbing fixtures on new roughing,  non -gas cooking and water heater as per plan.</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>EDISON</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>PAUL</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>40</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1720 VILLAGE LANE, Queens</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>MOTT CENTER LLC</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2940</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Q01350388-I1</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>INSTALLATION OF AN ILLUMINATED BUSINESS ACCESSORY SIGN. NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>JIN HWAN</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>CHO</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>40</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Alteration</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>166 WEST   18 STREET, Manhattan</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Douglas Elliman Property Management</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G65" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>363834</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>M01389555-I1</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>INTERIOR RENOVATION OF PHB (PENTHOUSE) APT, REMOVAL OF NON-LOAD BEARING PARTITIONS, ERECTION OF NEW NON-LOAD BEARING WALLS, FINISHES, MILLWORK, PAINTING, FLOORING AND SANDING WORK. ALL AS PER PLANS AND APPLICATIONS. NO CHANGE IN USE, EGRESS OR OCCUPANCY.</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Abdallah</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Elcherbini</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
         <v>0</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>4107 OCEAN AVENUE, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>SELF</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G66" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>480984</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>B00548726-P3</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>PROVIDING VERTICAL AND HORIZONTAL ENLARGEMENTS TO ENLARGE EXISTING TWO FAMILY RESIDENCE TO MAXIMUM PERMITTED FLOOR AREA.</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>IULIA</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>RATA</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>0</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>461 MACON STREET, Brooklyn</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G67" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>53600</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>B01233523-S1</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>FILING GAS &amp; PLUMBING WORK ON EXISTING 2 1/2 STORY BUILDING IN CONJUNCTION WITH JOB NO. B01233523-I1.  NO CHANGE IN USE, OCCUPANCY AND MEANS OF EGRESS IS INVOLVED UNDER THIS APPLICATION</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Feng</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Zhang</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>0</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Alteration CO</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>83-36 252 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Pending CPE/ACPE Assignment</t>
+        </is>
+      </c>
+      <c r="G68" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>66445</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Q01444508-I1</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>EXISTING ONE FAMILY  DWELLING UNIT   TO ADD NEW  2ND FLOOR VERTICAL EXTENSION AND KEEP ONE FAMILY DWELLING UNIT TO OBTAIN NEW CERTIFICATE OF OCCUPANCY (CO).</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>KARTIK</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>CHANDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>0</v>
+      </c>
+      <c r="B69" t="inlineStr">
         <is>
           <t>ALT-CO - New Building with Existing Elements to Remain</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>27-12 2 STREET, Queens</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>77-02GAR PITKIN AVENUE, Queens</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
         <is>
           <t>Queens</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>star dust</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="G21" s="1" t="n">
-        <v>46249</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Q01446395-I1</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>dd</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Aimarana</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>104</t>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Q01294623-P1</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>APPLICATION FILING TO REPAIR EXISTING GARAGE AS PER PLAN TO OBTAIN CERTIFICATE OF OCCUPANCY FOR TWO (2) ACCESSORY CAR GARAGE.</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Alauddin</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>0</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ALT-CO - New Building with Existing Elements to Remain</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>67-45 169 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Pending Prof Cert QA Assignment</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Q01446486-S2</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>INSTALL 8' TEMPORARY CONSTRUCTION FENCE AT THE ABOVE ADDRESS</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>KAI</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>HUANG</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>0</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ALT-CO - New Building with Existing Elements to Remain</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>67-45 169 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G71" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Q01446486-S1</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>FILE SOE IN CONJUNCTION WITH JOB#Q01446486</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>KAI</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>HUANG</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>0</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ALT-CO - New Building with Existing Elements to Remain</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>73-70 136 STREET, Queens</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Pending Plan Examiner Assignment</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Q01417905-S1</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>INSTALL SOE IN CONJUNCTION WITH JOB#Q01417905</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>XIAOHONG</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>ZHAO</t>
         </is>
       </c>
     </row>

</xml_diff>